<commit_message>
Add 20 unsold ASINs with cover images, updated categories (Notebook added)
</commit_message>
<xml_diff>
--- a/books_master_120.xlsx
+++ b/books_master_120.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4593,7 +4593,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Notebook</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4765,6 +4765,1046 @@
       <c r="J83" s="2" t="inlineStr">
         <is>
           <t>fish_kids_coloring.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Bugs Coloring Book For Kids</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>B0CMLVJFDH</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CMLVJFDH</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CMLVJFDH</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CMLVJFDH</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CMLVJFDH</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Build your Kids Creativity and ImaginationBetween the ages of 1 and 4 your child starts developing their creativity and imagination, with this book they can start seeing real world creations infront of their eyes. They start using different colors which help stimulate their creativity.70+ Amazing Bu</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>bugs_kids_coloring.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Bugs Coloring Book For Kids</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>B0CPQ254ZQ</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CPQ254ZQ</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CPQ254ZQ</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CPQ254ZQ</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CPQ254ZQ</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>Build your Kids Creativity and ImaginationBetween the ages of 1 and 4 your child starts developing their creativity and imagination, with this book they can start seeing real world creations infront of their eyes. They start using different colors which help stimulate their creativity.70+ Amazing Bu</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>bugs_kids_coloring_1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Bugs Coloring Book For Toddlers</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>B0CPQ36KFV</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CPQ36KFV</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CPQ36KFV</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CPQ36KFV</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CPQ36KFV</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>This is your Childs first experience expressing their creativity.Toddlers and Preschoolers will love this book full of Bugs coloring pagesStart showing creativity at an early age with a love for coloringProduce creative leaders for tomorrow new ageUse as a learning and teaching tool for Preschoolers</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>bugs_toddler_coloring_1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Christmas Recipe Book For Kids</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>B0BQ5DJ38H</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BQ5DJ38H</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BQ5DJ38H</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BQ5DJ38H</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BQ5DJ38H</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Have you ever just wanted a place to document those personal, family recipes from Mom or Grandma?Now you can do that in one easy to find book.Simple book for all those who love cooking and would like to document their recipes for later use.Can be personalized to reflect the users taste and personal </t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>kids_recipe_book_2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Christmas Recipe Book For Men</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>B0BQ5DRJW7</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BQ5DRJW7</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BQ5DRJW7</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BQ5DRJW7</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BQ5DRJW7</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Adult</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Have you ever just wanted a place to document those personal, family recipes from Mom or Grandma?Now you can do that in one easy to find book.Simple book for all those who love cooking and would like to document their recipes for later use.Can be personalized to reflect the users taste and personal </t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>christmas_recipe_men.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Christmas Recipe Book For Women</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>B0BQ5DRV19</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BQ5DRV19</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BQ5DRV19</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BQ5DRV19</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BQ5DRV19</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Adult</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Have you ever just wanted a place to document those personal, family recipes from Mom or Grandma?Now you can do that in one easy to find book.Simple book for all those who love cooking and would like to document their recipes for later use.Can be personalized to reflect the users taste and personal </t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>christmas_recipe_women.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Cute Hamster Coloring Book For Kids</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>B0CJL9SZN3</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CJL9SZN3</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CJL9SZN3</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CJL9SZN3</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CJL9SZN3</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Build your Kids Creativity and ImaginationBetween the ages of 1 and 4 your child starts developing their creativity and imagination, with this book they can start seeing real world creations infront of their eyes. They start using different colors which help stimulate their creativity.70+ Amazing Cu</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>cute_hamster_kids_coloring.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Cute Hamster Coloring Book For Toddlers</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>B0CJLLLV13</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CJLLLV13</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CJLLLV13</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CJLLLV13</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CJLLLV13</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>This is your Childs first experience expressing their creativity.Toddlers and Preschoolers will love this book full of Cute Hamster coloring pagesStart showing creativity at an early age with a love for coloringProduce creative leaders for tomorrow new ageUse as a learning and teaching tool for Pres</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>cute_hamster_toddler_coloring.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Daily Gratitude Journal For Kids</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>B0BKRWYDH8</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BKRWYDH8</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BKRWYDH8</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BKRWYDH8</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BKRWYDH8</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>Daily expressions of gratitude can improve one’s outlook on life. This beautiful gratitude Journal starts of with an inspiring bible verse designed to be a constant daily reminder to be grateful, It also provides space to record what you are thankful for on a daily basis in addition your prayers and</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>gratitude_kids.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Easter Recipe Book For Men</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>B0BTP1TXNP</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BTP1TXNP</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BTP1TXNP</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BTP1TXNP</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BTP1TXNP</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>Have you ever just wanted a place to write all those personal, family recipes from Mom or Grandma? Now you can do that in one easy to find kids book. Simple book for all those kids and youngones who love cooking and would like to save their recipes for later reading. Can be personalized to reflect t</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>easter_recipe_men.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Easter Recipe Book For Women</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>B0BTP1TXN9</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BTP1TXN9</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BTP1TXN9</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BTP1TXN9</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BTP1TXN9</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>Have you ever just wanted a place to write all those personal, family recipes from Mom or Grandma? Now you can do that in one easy to find kids book. Simple book for all those kids and youngones who love cooking and would like to save their recipes for later reading. Can be personalized to reflect t</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>easter_recipe_women.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Fun Fall Coloring Book For Kids</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>B0BR9DQGVM</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BR9DQGVM</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BR9DQGVM</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BR9DQGVM</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BR9DQGVM</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>Build your Kids Creativity and ImaginationBetween the ages of 1 and 4 your child starts developing their creativity and imagination, with this book they can start seeing real world creations infront of their eyes. They start using different colors which help stimulate their creativity.70+ Amazing Fu</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>fun_fall_kids_coloring.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Music Composition Notebook</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>B0CJKTT4M5</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CJKTT4M5</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CJKTT4M5</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CJKTT4M5</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CJKTT4M5</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Adult</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>Document your musical musings with this notebook.Each book is 8.5" x 11" and features 12 staves of printed music paper format on each sheet.110 pages of blank music manuscript on thick white paper</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>music_composition_1.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Music Composition Notebook</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>B0CJL3GJ6B</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CJL3GJ6B</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CJL3GJ6B</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CJL3GJ6B</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CJL3GJ6B</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Adult</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>Document your musical musings with this notebook.Each book is 8.5" x 11" and features 12 staves of printed music paper format on each sheet.110 pages of blank music manuscript on thick white paper</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>music_composition_2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Music Composition Notebook</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>B0CJL3VPYL</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CJL3VPYL</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CJL3VPYL</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CJL3VPYL</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CJL3VPYL</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Adult</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>Document your musical musings with this notebook.Each book is 8.5" x 11" and features 12 staves of printed music paper format on each sheet.110 pages of blank music manuscript on thick white paper</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>music_composition_3.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>My Easter Recipes From Mom</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>B0BTNSM73N</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BTNSM73N</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BTNSM73N</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BTNSM73N</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BTNSM73N</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>Have you ever just wanted a place to write all those personal, family recipes from Mom or Grandma? Now you can do that in one easy to find kids book. Simple book for all those kids and youngones who love cooking and would like to save their recipes for later reading. Can be personalized to reflect t</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>easter_recipe_mom.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>My Easter Recipes From GrandMa</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>B0BTP1WNLD</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BTP1WNLD</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BTP1WNLD</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BTP1WNLD</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BTP1WNLD</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>Have you ever just wanted a place to write all those personal, family recipes from Mom or Grandma? Now you can do that in one easy to find kids book. Simple book for all those kids and youngones who love cooking and would like to save their recipes for later reading. Can be personalized to reflect t</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>easter_recipe_grandma.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>My Favorite Christmas Recipes</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>B0BTNSL7LS</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BTNSL7LS</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BTNSL7LS</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BTNSL7LS</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BTNSL7LS</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Cookbook</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>Have you ever just wanted a place to write all those personal, family recipes from Mom or Grandma? Now you can do that in one easy to find kids book. Simple book for all those kids and youngones who love cooking and would like to save their recipes for later reading. Can be personalized to reflect t</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>christmas_recipe_book.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Panda Coloring Book For Kids</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>B0CQST5VSJ</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CQST5VSJ</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0CQST5VSJ</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0CQST5VSJ</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0CQST5VSJ</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>Build your Kids Creativity and ImaginationBetween the ages of 1 and 4 your child starts developing their creativity and imagination, with this book they can start seeing real world creations infront of their eyes. They start using different colors which help stimulate their creativity.70+ Amazing Pa</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>panda_kids_coloring.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Spring Flowers Coloring Book For Kids</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>B0BR996VVN</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0BR996VVN</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.co.uk/dp/B0BR996VVN</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0BR996VVN</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.au/dp/B0BR996VVN</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Coloring Book</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>Build your Kids Creativity and ImaginationBetween the ages of 1 and 4 your child starts developing their creativity and imagination, with this book they can start seeing real world creations infront of their eyes. They start using different colors which help stimulate their creativity.70+ Amazing Sp</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>spring_flowers_kids_coloring.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scrape real Amazon prices for all 102 books + add Price column to spreadsheet
</commit_message>
<xml_diff>
--- a/books_master_120.xlsx
+++ b/books_master_120.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -503,6 +503,11 @@
           <t>Cover_Filename</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Price_USD</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -555,6 +560,9 @@
           <t>dinosaur_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K2" t="n">
+        <v>11.48</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -607,6 +615,9 @@
           <t>dinosaur_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K3" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -659,6 +670,9 @@
           <t>birds_coloring.jpg</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>10.99</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -711,6 +725,9 @@
           <t>sermon_notes_journal_women.jpg</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -763,6 +780,9 @@
           <t>prayer_journal_women.jpg</t>
         </is>
       </c>
+      <c r="K6" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -815,6 +835,9 @@
           <t>spider_coloring_kids.jpg</t>
         </is>
       </c>
+      <c r="K7" t="n">
+        <v>11.48</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -867,6 +890,9 @@
           <t>spider_coloring_toddler.jpg</t>
         </is>
       </c>
+      <c r="K8" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -919,6 +945,9 @@
           <t>cute_pumpkin_toddler.jpg</t>
         </is>
       </c>
+      <c r="K9" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -971,6 +1000,9 @@
           <t>dinosaur_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K10" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1023,6 +1055,9 @@
           <t>kids_recipe_book.jpg</t>
         </is>
       </c>
+      <c r="K11" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1075,6 +1110,9 @@
           <t>sermon_notes_men.jpg</t>
         </is>
       </c>
+      <c r="K12" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1127,6 +1165,9 @@
           <t>prayer_teen_boys.jpg</t>
         </is>
       </c>
+      <c r="K13" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1179,6 +1220,9 @@
           <t>owl_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K14" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1231,6 +1275,9 @@
           <t>toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K15" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1283,6 +1330,9 @@
           <t>recipe_book.jpg</t>
         </is>
       </c>
+      <c r="K16" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1335,6 +1385,9 @@
           <t>recipe_book_write_your_own.jpg</t>
         </is>
       </c>
+      <c r="K17" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1387,6 +1440,9 @@
           <t>pumpkin_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K18" t="n">
+        <v>11.48</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1439,6 +1495,9 @@
           <t>cute_bunny_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K19" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1491,6 +1550,9 @@
           <t>christmas_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K20" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1543,6 +1605,9 @@
           <t>prayer_teen_girls.jpg</t>
         </is>
       </c>
+      <c r="K21" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1595,6 +1660,9 @@
           <t>butterfly_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K22" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1647,6 +1715,9 @@
           <t>cute_farm_animals_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K23" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1699,6 +1770,9 @@
           <t>cute_kitty_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K24" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1751,6 +1825,9 @@
           <t>first_abc_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K25" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1803,6 +1880,9 @@
           <t>dinosaur_kids_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K26" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1855,6 +1935,9 @@
           <t>fun_thanksgiving_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K27" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1907,6 +1990,9 @@
           <t>sea_turtle_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K28" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1959,6 +2045,9 @@
           <t>christmas_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K29" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2011,6 +2100,9 @@
           <t>prayer_men.jpg</t>
         </is>
       </c>
+      <c r="K30" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2063,6 +2155,9 @@
           <t>cute_fox_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K31" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2115,6 +2210,9 @@
           <t>cute_kitty_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K32" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2167,6 +2265,9 @@
           <t>gratitude_teen_girls.jpg</t>
         </is>
       </c>
+      <c r="K33" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2219,6 +2320,9 @@
           <t>first_abc_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K34" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2271,6 +2375,9 @@
           <t>gratitude_men.jpg</t>
         </is>
       </c>
+      <c r="K35" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2323,6 +2430,9 @@
           <t>panda_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K36" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2375,6 +2485,9 @@
           <t>prayer_kids.jpg</t>
         </is>
       </c>
+      <c r="K37" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2427,6 +2540,9 @@
           <t>llama_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K38" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2479,6 +2595,9 @@
           <t>fun_animal_african_american_coloring.jpg</t>
         </is>
       </c>
+      <c r="K39" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2531,6 +2650,9 @@
           <t>toddler_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K40" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2583,6 +2705,9 @@
           <t>gratitude_teen_boys.jpg</t>
         </is>
       </c>
+      <c r="K41" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2635,6 +2760,9 @@
           <t>owl_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K42" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2687,6 +2815,9 @@
           <t>fun_animal_african_american_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K43" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2739,6 +2870,9 @@
           <t>easter_egg_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K44" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2791,6 +2925,9 @@
           <t>fun_animal_coloring.jpg</t>
         </is>
       </c>
+      <c r="K45" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2843,6 +2980,9 @@
           <t>toddler_coloring_2.jpg</t>
         </is>
       </c>
+      <c r="K46" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2895,6 +3035,9 @@
           <t>gratitude_men_1.jpg</t>
         </is>
       </c>
+      <c r="K47" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2947,6 +3090,9 @@
           <t>cute_bunny_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K48" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2999,6 +3145,9 @@
           <t>spring_flowers_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K49" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3051,6 +3200,9 @@
           <t>humming_bird_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K50" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3103,6 +3255,9 @@
           <t>bugs_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K51" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3155,6 +3310,9 @@
           <t>kisa_recipe_book.jpg</t>
         </is>
       </c>
+      <c r="K52" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3207,6 +3365,9 @@
           <t>fun_animal_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K53" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3259,6 +3420,9 @@
           <t>cute_fox_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K54" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3311,6 +3475,9 @@
           <t>toddler_coloring_3.jpg</t>
         </is>
       </c>
+      <c r="K55" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3363,6 +3530,9 @@
           <t>fun_sealife_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K56" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3415,6 +3585,9 @@
           <t>cute_puppy_dog_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K57" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3467,6 +3640,9 @@
           <t>cute_farm_animals_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K58" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3519,6 +3695,9 @@
           <t>kids_recipe_book_1.jpg</t>
         </is>
       </c>
+      <c r="K59" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3571,6 +3750,9 @@
           <t>christmas_recipe.jpg</t>
         </is>
       </c>
+      <c r="K60" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3623,6 +3805,9 @@
           <t>birds_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K61" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3675,6 +3860,9 @@
           <t>birds_coloring_2.jpg</t>
         </is>
       </c>
+      <c r="K62" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3727,6 +3915,9 @@
           <t>cute_puppy_dog_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K63" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3779,6 +3970,9 @@
           <t>christmas_recipe_mom.jpg</t>
         </is>
       </c>
+      <c r="K64" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3831,6 +4025,9 @@
           <t>ladybug_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K65" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3883,6 +4080,9 @@
           <t>llama_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K66" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3935,6 +4135,9 @@
           <t>dinosaur_kids_coloring_2.jpg</t>
         </is>
       </c>
+      <c r="K67" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3987,6 +4190,9 @@
           <t>easter_egg_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K68" t="n">
+        <v>10.98</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4039,6 +4245,9 @@
           <t>humming_bird_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K69" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4091,6 +4300,9 @@
           <t>sea_turtle_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K70" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4143,6 +4355,9 @@
           <t>ladybug_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K71" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4195,6 +4410,9 @@
           <t>birds_coloring_3.jpg</t>
         </is>
       </c>
+      <c r="K72" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4247,6 +4465,9 @@
           <t>birds_coloring_4.jpg</t>
         </is>
       </c>
+      <c r="K73" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4299,6 +4520,9 @@
           <t>fun_halloween_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K74" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4351,6 +4575,9 @@
           <t>first_abc_kids_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K75" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4403,6 +4630,9 @@
           <t>cute_kitty_kids_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K76" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4455,6 +4685,9 @@
           <t>christmas_recipe_grandma.jpg</t>
         </is>
       </c>
+      <c r="K77" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4507,6 +4740,9 @@
           <t>fun_fall_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K78" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4559,6 +4795,9 @@
           <t>butterfly_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K79" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4611,6 +4850,9 @@
           <t>music_composition.jpg</t>
         </is>
       </c>
+      <c r="K80" t="n">
+        <v>7.98</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4663,6 +4905,9 @@
           <t>sea_turtle_kids_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K81" t="n">
+        <v>14.98</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4715,6 +4960,9 @@
           <t>fish_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K82" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4767,6 +5015,9 @@
           <t>fish_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K83" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4819,6 +5070,9 @@
           <t>bugs_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K84" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4871,6 +5125,9 @@
           <t>bugs_kids_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K85" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4923,6 +5180,9 @@
           <t>bugs_toddler_coloring_1.jpg</t>
         </is>
       </c>
+      <c r="K86" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4975,6 +5235,9 @@
           <t>kids_recipe_book_2.jpg</t>
         </is>
       </c>
+      <c r="K87" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5027,6 +5290,9 @@
           <t>christmas_recipe_men.jpg</t>
         </is>
       </c>
+      <c r="K88" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5079,6 +5345,9 @@
           <t>christmas_recipe_women.jpg</t>
         </is>
       </c>
+      <c r="K89" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5131,6 +5400,9 @@
           <t>cute_hamster_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K90" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5183,6 +5455,9 @@
           <t>cute_hamster_toddler_coloring.jpg</t>
         </is>
       </c>
+      <c r="K91" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5235,6 +5510,9 @@
           <t>gratitude_kids.jpg</t>
         </is>
       </c>
+      <c r="K92" t="n">
+        <v>9.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5287,6 +5565,9 @@
           <t>easter_recipe_men.jpg</t>
         </is>
       </c>
+      <c r="K93" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5339,6 +5620,9 @@
           <t>easter_recipe_women.jpg</t>
         </is>
       </c>
+      <c r="K94" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5391,6 +5675,9 @@
           <t>fun_fall_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K95" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5443,6 +5730,9 @@
           <t>music_composition_1.jpg</t>
         </is>
       </c>
+      <c r="K96" t="n">
+        <v>7.98</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5495,6 +5785,9 @@
           <t>music_composition_2.jpg</t>
         </is>
       </c>
+      <c r="K97" t="n">
+        <v>7.98</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5547,6 +5840,9 @@
           <t>music_composition_3.jpg</t>
         </is>
       </c>
+      <c r="K98" t="n">
+        <v>7.98</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5599,6 +5895,9 @@
           <t>easter_recipe_mom.jpg</t>
         </is>
       </c>
+      <c r="K99" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5651,6 +5950,9 @@
           <t>easter_recipe_grandma.jpg</t>
         </is>
       </c>
+      <c r="K100" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -5703,6 +6005,9 @@
           <t>christmas_recipe_book.jpg</t>
         </is>
       </c>
+      <c r="K101" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5755,6 +6060,9 @@
           <t>panda_kids_coloring.jpg</t>
         </is>
       </c>
+      <c r="K102" t="n">
+        <v>10.48</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5806,6 +6114,9 @@
         <is>
           <t>spring_flowers_kids_coloring.jpg</t>
         </is>
+      </c>
+      <c r="K103" t="n">
+        <v>10.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>